<commit_message>
Project the gambling duty bases with OBR Table 4.10
Each of the fifteen gambling inputs declares the uprating index of its
duty, and dataset projection grows it by the same series. The series come
from RECEIPTS_SERIES_SPECS: the OBR's October 2026 betting and gaming
forecast breakdown (receipts Table 4.10), after HMRC's 2024-25 and
2025-26 receipts, less Autumn Budget 2026 measure 56 for Machine Games
Duty, divided by the rates the model charges. The model then applies the
April 2026 Remote Gaming Duty and April 2027 remote betting rate rises
once, not twice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/policyengine_uk/tests/fixtures/obr_receipts/obr_efo_march_2026_receipts.xlsx
+++ b/policyengine_uk/tests/fixtures/obr_receipts/obr_efo_march_2026_receipts.xlsx
@@ -18,6 +18,7 @@
     <ns0:sheet name="3.2" sheetId="194" ns7:id="rId3"/>
     <ns0:sheet name="3.7" sheetId="204" ns7:id="rId8"/>
     <ns0:sheet name="3.8" sheetId="192" ns7:id="rId9"/>
+    <ns0:sheet name="3.10" sheetId="261" ns7:id="rId11"/>
   </ns0:sheets>
   <ns0:definedNames>
     <ns0:definedName name="________tab3" localSheetId="18">!#REF!</ns0:definedName>
@@ -4045,6 +4046,287 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{270C67AD-4C14-4065-AB23-9509227752CC}">
+  <sheetPr codeName="Sheet30">
+    <tabColor theme="4" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="354" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" style="354" customWidth="1"/>
+    <col min="3" max="8" width="10" style="354" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="354"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="33.75" customHeight="1" thickBot="1">
+      <c r="A1" s="339" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" thickBot="1">
+      <c r="B2" s="563" t="s">
+        <v>307</v>
+      </c>
+      <c r="C2" s="564"/>
+      <c r="D2" s="564"/>
+      <c r="E2" s="564"/>
+      <c r="F2" s="564"/>
+      <c r="G2" s="564"/>
+      <c r="H2" s="565"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="B3" s="343"/>
+      <c r="C3" s="561" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="561"/>
+      <c r="E3" s="561"/>
+      <c r="F3" s="561"/>
+      <c r="G3" s="561"/>
+      <c r="H3" s="562"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="B4" s="269"/>
+      <c r="C4" s="559" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="559"/>
+      <c r="E4" s="559"/>
+      <c r="F4" s="559"/>
+      <c r="G4" s="559"/>
+      <c r="H4" s="560"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="B5" s="269"/>
+      <c r="C5" s="264" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="264" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="264" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" s="264" t="s">
+        <v>122</v>
+      </c>
+      <c r="G5" s="264" t="s">
+        <v>161</v>
+      </c>
+      <c r="H5" s="340" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B6" s="272" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="356">
+        <v>3.7972275673045832</v>
+      </c>
+      <c r="D6" s="356">
+        <v>4.7977750909717853</v>
+      </c>
+      <c r="E6" s="356">
+        <v>5.1562161360302587</v>
+      </c>
+      <c r="F6" s="356">
+        <v>5.3562538432896201</v>
+      </c>
+      <c r="G6" s="356">
+        <v>5.5388440890340274</v>
+      </c>
+      <c r="H6" s="357">
+        <v>5.6840393787403398</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B7" s="273" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="265"/>
+      <c r="D7" s="265"/>
+      <c r="E7" s="265"/>
+      <c r="F7" s="265"/>
+      <c r="G7" s="265"/>
+      <c r="H7" s="267"/>
+    </row>
+    <row r="8" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B8" s="276" t="s">
+        <v>253</v>
+      </c>
+      <c r="C8" s="265">
+        <v>1.312896340550628</v>
+      </c>
+      <c r="D8" s="265">
+        <v>2.3161989343494422</v>
+      </c>
+      <c r="E8" s="265">
+        <v>2.4150072286414543</v>
+      </c>
+      <c r="F8" s="265">
+        <v>2.5371533459117006</v>
+      </c>
+      <c r="G8" s="265">
+        <v>2.6491836780604188</v>
+      </c>
+      <c r="H8" s="267">
+        <v>2.7306035741759453</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B9" s="276" t="s">
+        <v>251</v>
+      </c>
+      <c r="C9" s="265">
+        <v>0.96112324524158754</v>
+      </c>
+      <c r="D9" s="265">
+        <v>1.0085681777616253</v>
+      </c>
+      <c r="E9" s="265">
+        <v>1.0341499168843902</v>
+      </c>
+      <c r="F9" s="265">
+        <v>1.0590432874187228</v>
+      </c>
+      <c r="G9" s="265">
+        <v>1.0900246600358603</v>
+      </c>
+      <c r="H9" s="267">
+        <v>1.1149544752961229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B10" s="276" t="s">
+        <v>252</v>
+      </c>
+      <c r="C10" s="265">
+        <v>0.6730606094724928</v>
+      </c>
+      <c r="D10" s="265">
+        <v>0.69778590690050302</v>
+      </c>
+      <c r="E10" s="265">
+        <v>0.92838385767587883</v>
+      </c>
+      <c r="F10" s="265">
+        <v>0.97136805940446491</v>
+      </c>
+      <c r="G10" s="265">
+        <v>1.0025732078128275</v>
+      </c>
+      <c r="H10" s="267">
+        <v>1.0340445095421</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B11" s="276" t="s">
+        <v>254</v>
+      </c>
+      <c r="C11" s="265">
+        <v>0.62861473757399211</v>
+      </c>
+      <c r="D11" s="265">
+        <v>0.60942497205580215</v>
+      </c>
+      <c r="E11" s="265">
+        <v>0.61520645642337479</v>
+      </c>
+      <c r="F11" s="265">
+        <v>0.62456887662211369</v>
+      </c>
+      <c r="G11" s="265">
+        <v>0.63433996958674899</v>
+      </c>
+      <c r="H11" s="267">
+        <v>0.64884821213584543</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B12" s="276" t="s">
+        <v>255</v>
+      </c>
+      <c r="C12" s="265">
+        <v>0.19430257515489857</v>
+      </c>
+      <c r="D12" s="265">
+        <v>0.16152282987590175</v>
+      </c>
+      <c r="E12" s="265">
+        <v>0.15895769101927501</v>
+      </c>
+      <c r="F12" s="265">
+        <v>0.15957236791081084</v>
+      </c>
+      <c r="G12" s="265">
+        <v>0.15798637304398647</v>
+      </c>
+      <c r="H12" s="267">
+        <v>0.15076269408490447</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="13.5" customHeight="1">
+      <c r="B13" s="276" t="s">
+        <v>256</v>
+      </c>
+      <c r="C13" s="265">
+        <v>2.3468950845847075E-2</v>
+      </c>
+      <c r="D13" s="265">
+        <v>1.3709635323819284E-8</v>
+      </c>
+      <c r="E13" s="265">
+        <v>3.7090695150306794E-8</v>
+      </c>
+      <c r="F13" s="265">
+        <v>3.8199404950839866E-8</v>
+      </c>
+      <c r="G13" s="265">
+        <v>3.8960655399193704E-8</v>
+      </c>
+      <c r="H13" s="267">
+        <v>4.0149031057811823E-8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="13.5" customHeight="1" thickBot="1">
+      <c r="B14" s="277" t="s">
+        <v>257</v>
+      </c>
+      <c r="C14" s="341">
+        <v>3.7611084651374858E-3</v>
+      </c>
+      <c r="D14" s="341">
+        <v>4.2742563188752965E-3</v>
+      </c>
+      <c r="E14" s="341">
+        <v>4.5109482951906227E-3</v>
+      </c>
+      <c r="F14" s="341">
+        <v>4.547867822402683E-3</v>
+      </c>
+      <c r="G14" s="341">
+        <v>4.7361615335291072E-3</v>
+      </c>
+      <c r="H14" s="342">
+        <v>4.825873356391056E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="B2:H2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A1" location="Contents!A1" display="Back to contents" xr:uid="{8326E600-4ACE-4B09-A201-6586B1299CBB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{657582D5-BD3B-4482-82A3-154823C755A5}">
   <sheetPr codeName="Sheet4">

</xml_diff>